<commit_message>
fix: clear invalid articy template headers in Fishing import
</commit_message>
<xml_diff>
--- a/stories/fishing/articy/fishing-import.xlsx
+++ b/stories/fishing/articy/fishing-import.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Entities" sheetId="1" r:id="Rff9b8946922e4a83"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Flow Fragments" sheetId="2" r:id="Rd1b3ec8604614e8a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Global Variables" sheetId="3" r:id="R4034a5a8107f4a62"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Entities" sheetId="1" r:id="Recc796beceee4266"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Flow Fragments" sheetId="2" r:id="R1f9e70c64bdd4a07"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Global Variables" sheetId="3" r:id="R834c05c9d9544246"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -25,9 +25,6 @@
   </x:si>
   <x:si>
     <x:t xml:space="preserve">Template Name:</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">1</x:t>
   </x:si>
   <x:si>
     <x:t xml:space="preserve">Project Guid:</x:t>
@@ -531,19 +528,17 @@
       <x:c r="A2" s="1" t="s">
         <x:v>4</x:v>
       </x:c>
-      <x:c r="B2" s="1" t="s">
+      <x:c r="B2" s="1"/>
+      <x:c r="C2" s="1" t="s">
         <x:v>5</x:v>
       </x:c>
-      <x:c r="C2" s="1" t="s">
+      <x:c r="D2" s="1" t="s">
         <x:v>6</x:v>
-      </x:c>
-      <x:c r="D2" s="1" t="s">
-        <x:v>7</x:v>
       </x:c>
     </x:row>
     <x:row r="3" s="1" customFormat="1">
       <x:c r="A3" s="1" t="s">
-        <x:v>8</x:v>
+        <x:v>7</x:v>
       </x:c>
       <x:c r="B3" s="3">
         <x:v>46305.6125689236</x:v>
@@ -551,34 +546,34 @@
     </x:row>
     <x:row r="4" s="2" customFormat="1">
       <x:c r="A4" s="2" t="s">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="B4" s="2" t="s">
         <x:v>9</x:v>
       </x:c>
-      <x:c r="B4" s="2" t="s">
+      <x:c r="C4" s="2" t="s">
         <x:v>10</x:v>
       </x:c>
-      <x:c r="C4" s="2" t="s">
+      <x:c r="D4" s="2" t="s">
         <x:v>11</x:v>
       </x:c>
-      <x:c r="D4" s="2" t="s">
+      <x:c r="E4" s="2" t="s">
         <x:v>12</x:v>
       </x:c>
-      <x:c r="E4" s="2" t="s">
+      <x:c r="F4" s="2" t="s">
         <x:v>13</x:v>
       </x:c>
-      <x:c r="F4" s="2" t="s">
+      <x:c r="G4" s="2" t="s">
         <x:v>14</x:v>
       </x:c>
-      <x:c r="G4" s="2" t="s">
+      <x:c r="H4" s="2" t="s">
         <x:v>15</x:v>
       </x:c>
-      <x:c r="H4" s="2" t="s">
+      <x:c r="I4" s="2" t="s">
         <x:v>16</x:v>
       </x:c>
-      <x:c r="I4" s="2" t="s">
+      <x:c r="J4" s="2" t="s">
         <x:v>17</x:v>
-      </x:c>
-      <x:c r="J4" s="2" t="s">
-        <x:v>18</x:v>
       </x:c>
     </x:row>
     <x:row r="5" ht="110" customHeight="1">
@@ -725,7 +720,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="B1" s="1" t="s">
-        <x:v>19</x:v>
+        <x:v>18</x:v>
       </x:c>
       <x:c r="C1" s="1" t="s">
         <x:v>2</x:v>
@@ -738,19 +733,17 @@
       <x:c r="A2" s="1" t="s">
         <x:v>4</x:v>
       </x:c>
-      <x:c r="B2" s="1" t="s">
+      <x:c r="B2" s="1"/>
+      <x:c r="C2" s="1" t="s">
         <x:v>5</x:v>
       </x:c>
-      <x:c r="C2" s="1" t="s">
+      <x:c r="D2" s="1" t="s">
         <x:v>6</x:v>
-      </x:c>
-      <x:c r="D2" s="1" t="s">
-        <x:v>7</x:v>
       </x:c>
     </x:row>
     <x:row r="3" s="1" customFormat="1">
       <x:c r="A3" s="1" t="s">
-        <x:v>8</x:v>
+        <x:v>7</x:v>
       </x:c>
       <x:c r="B3" s="3">
         <x:v>46305.6125704051</x:v>
@@ -758,34 +751,34 @@
     </x:row>
     <x:row r="4" s="2" customFormat="1">
       <x:c r="A4" s="2" t="s">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="B4" s="2" t="s">
         <x:v>9</x:v>
       </x:c>
-      <x:c r="B4" s="2" t="s">
+      <x:c r="C4" s="2" t="s">
         <x:v>10</x:v>
       </x:c>
-      <x:c r="C4" s="2" t="s">
+      <x:c r="D4" s="2" t="s">
         <x:v>11</x:v>
       </x:c>
-      <x:c r="D4" s="2" t="s">
+      <x:c r="E4" s="2" t="s">
         <x:v>12</x:v>
       </x:c>
-      <x:c r="E4" s="2" t="s">
+      <x:c r="F4" s="2" t="s">
         <x:v>13</x:v>
       </x:c>
-      <x:c r="F4" s="2" t="s">
+      <x:c r="G4" s="2" t="s">
         <x:v>14</x:v>
       </x:c>
-      <x:c r="G4" s="2" t="s">
+      <x:c r="H4" s="2" t="s">
         <x:v>15</x:v>
       </x:c>
-      <x:c r="H4" s="2" t="s">
+      <x:c r="I4" s="2" t="s">
         <x:v>16</x:v>
       </x:c>
-      <x:c r="I4" s="2" t="s">
+      <x:c r="J4" s="2" t="s">
         <x:v>17</x:v>
-      </x:c>
-      <x:c r="J4" s="2" t="s">
-        <x:v>18</x:v>
       </x:c>
     </x:row>
     <x:row r="5" ht="110" customHeight="1">
@@ -1914,13 +1907,13 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="C1" s="1" t="s">
-        <x:v>20</x:v>
+        <x:v>19</x:v>
       </x:c>
     </x:row>
     <x:row r="2" s="1" customFormat="1"/>
     <x:row r="3" s="1" customFormat="1">
       <x:c r="B3" s="1" t="s">
-        <x:v>8</x:v>
+        <x:v>7</x:v>
       </x:c>
       <x:c r="C3" s="3">
         <x:v>46305.6125708796</x:v>
@@ -1928,22 +1921,22 @@
     </x:row>
     <x:row r="4" s="2" customFormat="1">
       <x:c r="A4" s="2" t="s">
-        <x:v>9</x:v>
+        <x:v>8</x:v>
       </x:c>
       <x:c r="B4" s="2" t="s">
+        <x:v>20</x:v>
+      </x:c>
+      <x:c r="C4" s="2" t="s">
         <x:v>21</x:v>
       </x:c>
-      <x:c r="C4" s="2" t="s">
+      <x:c r="D4" s="2" t="s">
         <x:v>22</x:v>
       </x:c>
-      <x:c r="D4" s="2" t="s">
+      <x:c r="E4" s="2" t="s">
         <x:v>23</x:v>
       </x:c>
-      <x:c r="E4" s="2" t="s">
+      <x:c r="F4" s="2" t="s">
         <x:v>24</x:v>
-      </x:c>
-      <x:c r="F4" s="2" t="s">
-        <x:v>25</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>